<commit_message>
The following objects were updated: IntegrationFlow, ScriptCollection, MessageMapping
</commit_message>
<xml_diff>
--- a/NewPackage/IntegrationFlow/Test_Flow/Documentation.xlsx
+++ b/NewPackage/IntegrationFlow/Test_Flow/Documentation.xlsx
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="77">
   <si>
     <t>Interface Details</t>
   </si>
@@ -212,7 +212,16 @@
     <t/>
   </si>
   <si>
-    <t>CPI IFlow Version 1.0.3, Figaf revision: 3</t>
+    <t>CPI IFlow Version 1.0.4, Figaf revision: 4</t>
+  </si>
+  <si>
+    <t>Sender</t>
+  </si>
+  <si>
+    <t>HTTPS</t>
+  </si>
+  <si>
+    <t>/new-test</t>
   </si>
   <si>
     <t>Integration Process</t>
@@ -263,7 +272,7 @@
     <t>Test_Flow iflow configuration.json</t>
   </si>
   <si>
-    <t>2026-07-26 23:02 PM</t>
+    <t>2026-07-31 09:07 AM</t>
   </si>
 </sst>
 </file>
@@ -1205,29 +1214,25 @@
       <c r="I4" s="2"/>
       <c r="J4" s="2"/>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A5" s="7"/>
-      <c r="B5" s="7"/>
-      <c r="C5" s="7"/>
-      <c r="D5" s="7"/>
+    <row r="5" ht="15.0" customHeight="true">
+      <c r="A5" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="B5" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="D5" s="7" t="s">
+        <v>59</v>
+      </c>
       <c r="E5" s="1"/>
       <c r="F5" s="1"/>
       <c r="G5" s="1"/>
       <c r="H5" s="1"/>
       <c r="I5" s="2"/>
       <c r="J5" s="2"/>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A6" s="1"/>
-      <c r="B6" s="1"/>
-      <c r="C6" s="1"/>
-      <c r="D6" s="1"/>
-      <c r="E6" s="1"/>
-      <c r="F6" s="1"/>
-      <c r="G6" s="1"/>
-      <c r="H6" s="1"/>
-      <c r="I6" s="2"/>
-      <c r="J6" s="2"/>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" s="1"/>
@@ -1613,42 +1618,42 @@
     </row>
     <row r="5" ht="15.0" customHeight="true">
       <c r="A5" s="7" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="B5" s="7" t="s">
         <v>55</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="E5" s="7" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="F5" s="9" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
     </row>
     <row r="6" ht="15.0" customHeight="true">
       <c r="A6" s="7" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="B6" s="7" t="s">
         <v>55</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="F6" s="9" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
     </row>
   </sheetData>
@@ -1711,36 +1716,36 @@
     </row>
     <row r="5" ht="15.0" customHeight="true">
       <c r="A5" s="7" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="C5" s="7" t="n">
         <v>1.0</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="E5" s="7" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
     </row>
     <row r="6" ht="15.0" customHeight="true">
       <c r="A6" s="7" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="C6" s="7" t="n">
         <v>2.0</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
     </row>
   </sheetData>
@@ -1792,13 +1797,13 @@
     </row>
     <row r="5" ht="15.0" customHeight="true">
       <c r="A5" s="7" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
The following objects were updated: IntegrationFlow
</commit_message>
<xml_diff>
--- a/NewPackage/IntegrationFlow/Test_Flow/Documentation.xlsx
+++ b/NewPackage/IntegrationFlow/Test_Flow/Documentation.xlsx
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="86">
   <si>
     <t>Interface Details</t>
   </si>
@@ -212,7 +212,7 @@
     <t/>
   </si>
   <si>
-    <t>CPI IFlow Version 1.0.4, Figaf revision: 4</t>
+    <t>CPI IFlow Version 1.0.5, Figaf revision: 5</t>
   </si>
   <si>
     <t>Sender</t>
@@ -224,6 +224,15 @@
     <t>/new-test</t>
   </si>
   <si>
+    <t>2026-07-31</t>
+  </si>
+  <si>
+    <t>daniel</t>
+  </si>
+  <si>
+    <t>REGRESSION</t>
+  </si>
+  <si>
     <t>Integration Process</t>
   </si>
   <si>
@@ -239,10 +248,22 @@
     <t>Start</t>
   </si>
   <si>
+    <t>CallActivity_5</t>
+  </si>
+  <si>
+    <t>2</t>
+  </si>
+  <si>
+    <t>callActivity</t>
+  </si>
+  <si>
+    <t>Groovy Script 1</t>
+  </si>
+  <si>
     <t>EndEvent_2</t>
   </si>
   <si>
-    <t>2</t>
+    <t>3</t>
   </si>
   <si>
     <t>endEvent</t>
@@ -272,7 +293,13 @@
     <t>Test_Flow iflow configuration.json</t>
   </si>
   <si>
-    <t>2026-07-31 09:07 AM</t>
+    <t>2026-07-31 10:37 AM</t>
+  </si>
+  <si>
+    <t>Script</t>
+  </si>
+  <si>
+    <t>script1.groovy</t>
   </si>
 </sst>
 </file>
@@ -1540,17 +1567,33 @@
         <v>30</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="5" ht="15.0" customHeight="true">
       <c r="A5" s="7"/>
       <c r="B5" s="7"/>
-      <c r="C5" s="7"/>
-      <c r="D5" s="7"/>
-      <c r="E5" s="7"/>
-      <c r="F5" s="7"/>
-      <c r="G5" s="7"/>
-      <c r="H5" s="7"/>
-      <c r="I5" s="7"/>
-      <c r="J5" s="7"/>
+      <c r="C5" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="D5" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="E5" s="7" t="s">
+        <v>62</v>
+      </c>
+      <c r="F5" s="7" t="n">
+        <v>2.0</v>
+      </c>
+      <c r="G5" s="7" t="n">
+        <v>2.0</v>
+      </c>
+      <c r="H5" s="7" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="I5" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="J5" s="7" t="n">
+        <v>0.0</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -1563,7 +1606,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" customWidth="true" width="19.42578125"/>
@@ -1618,42 +1661,62 @@
     </row>
     <row r="5" ht="15.0" customHeight="true">
       <c r="A5" s="7" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="B5" s="7" t="s">
         <v>55</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="E5" s="7" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="F5" s="9" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
     </row>
     <row r="6" ht="15.0" customHeight="true">
       <c r="A6" s="7" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="B6" s="7" t="s">
         <v>55</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="F6" s="9" t="s">
-        <v>68</v>
+        <v>71</v>
+      </c>
+    </row>
+    <row r="7" ht="15.0" customHeight="true">
+      <c r="A7" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="B7" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="C7" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="D7" s="7" t="s">
+        <v>73</v>
+      </c>
+      <c r="E7" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="F7" s="9" t="s">
+        <v>75</v>
       </c>
     </row>
   </sheetData>
@@ -1716,36 +1779,36 @@
     </row>
     <row r="5" ht="15.0" customHeight="true">
       <c r="A5" s="7" t="s">
-        <v>69</v>
+        <v>76</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>70</v>
+        <v>77</v>
       </c>
       <c r="C5" s="7" t="n">
         <v>1.0</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>71</v>
+        <v>78</v>
       </c>
       <c r="E5" s="7" t="s">
-        <v>72</v>
+        <v>79</v>
       </c>
     </row>
     <row r="6" ht="15.0" customHeight="true">
       <c r="A6" s="7" t="s">
-        <v>69</v>
+        <v>76</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>70</v>
+        <v>77</v>
       </c>
       <c r="C6" s="7" t="n">
         <v>2.0</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>73</v>
+        <v>80</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>72</v>
+        <v>79</v>
       </c>
     </row>
   </sheetData>
@@ -1759,7 +1822,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" customWidth="true" width="22.0"/>
@@ -1797,13 +1860,24 @@
     </row>
     <row r="5" ht="15.0" customHeight="true">
       <c r="A5" s="7" t="s">
-        <v>74</v>
+        <v>81</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>75</v>
+        <v>82</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>76</v>
+        <v>83</v>
+      </c>
+    </row>
+    <row r="6" ht="15.0" customHeight="true">
+      <c r="A6" s="7" t="s">
+        <v>84</v>
+      </c>
+      <c r="B6" s="7" t="s">
+        <v>85</v>
+      </c>
+      <c r="C6" s="7" t="s">
+        <v>83</v>
       </c>
     </row>
   </sheetData>

</xml_diff>